<commit_message>
problem: longest palindromic subString using bottom-up
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>date</t>
   </si>
@@ -169,6 +169,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/unique-paths-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longest Palindromic String</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/longest-palindromic-substring/description/</t>
   </si>
 </sst>
 </file>
@@ -981,7 +987,7 @@
       </c>
     </row>
     <row r="25" ht="14.25">
-      <c r="A25" s="3">
+      <c r="A25" s="1">
         <v>46056</v>
       </c>
       <c r="B25" t="s">
@@ -989,6 +995,17 @@
       </c>
       <c r="C25" s="2" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="A26" s="3">
+        <v>46056</v>
+      </c>
+      <c r="B26" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1016,6 +1033,7 @@
     <hyperlink r:id="rId21" ref="C23"/>
     <hyperlink r:id="rId22" ref="C24"/>
     <hyperlink r:id="rId23" ref="C25"/>
+    <hyperlink r:id="rId24" ref="C26"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: merge 2 sorted LLs
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>date</t>
   </si>
@@ -187,6 +187,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/interleaving-string/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merge 2 Sorted LL</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1038,7 @@
       </c>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="3">
+      <c r="A28" s="1">
         <v>46085</v>
       </c>
       <c r="B28" t="s">
@@ -1040,6 +1046,17 @@
       </c>
       <c r="C28" s="2" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="A29" s="3">
+        <v>46085</v>
+      </c>
+      <c r="B29" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1070,6 +1087,7 @@
     <hyperlink r:id="rId24" ref="C26"/>
     <hyperlink r:id="rId25" ref="C27"/>
     <hyperlink r:id="rId26" ref="C28"/>
+    <hyperlink r:id="rId27" ref="C29"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problems: detect cycles in a LL and remove nth node from end
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>date</t>
   </si>
@@ -193,6 +193,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/merge-two-sorted-lists/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linked List Cycle</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/linked-list-cycle/description/</t>
+  </si>
+  <si>
+    <t>DeleteNthLastNodeFromEnd</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
   </si>
 </sst>
 </file>
@@ -1049,7 +1061,7 @@
       </c>
     </row>
     <row r="29" ht="14.25">
-      <c r="A29" s="3">
+      <c r="A29" s="1">
         <v>46085</v>
       </c>
       <c r="B29" t="s">
@@ -1057,6 +1069,28 @@
       </c>
       <c r="C29" s="2" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="30" ht="14.25">
+      <c r="A30" s="1">
+        <v>46085</v>
+      </c>
+      <c r="B30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" ht="14.25">
+      <c r="A31" s="3">
+        <v>46085</v>
+      </c>
+      <c r="B31" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1088,6 +1122,8 @@
     <hyperlink r:id="rId25" ref="C27"/>
     <hyperlink r:id="rId26" ref="C28"/>
     <hyperlink r:id="rId27" ref="C29"/>
+    <hyperlink r:id="rId28" ref="C30"/>
+    <hyperlink r:id="rId29" ref="C31"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problems: add 2 nums (LL)
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t>date</t>
   </si>
@@ -205,6 +205,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">add 2 nos.</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/add-two-numbers/</t>
   </si>
 </sst>
 </file>
@@ -1083,7 +1089,7 @@
       </c>
     </row>
     <row r="31" ht="14.25">
-      <c r="A31" s="3">
+      <c r="A31" s="1">
         <v>46085</v>
       </c>
       <c r="B31" t="s">
@@ -1091,6 +1097,17 @@
       </c>
       <c r="C31" s="2" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="32" ht="14.25">
+      <c r="A32" s="3">
+        <v>46086</v>
+      </c>
+      <c r="B32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1124,6 +1141,7 @@
     <hyperlink r:id="rId27" ref="C29"/>
     <hyperlink r:id="rId28" ref="C30"/>
     <hyperlink r:id="rId29" ref="C31"/>
+    <hyperlink r:id="rId30" ref="C32"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: best time to buy and sell stocks 1,2 and 3
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>date</t>
   </si>
@@ -217,6 +217,24 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/edit-distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">best time to buy and sell stocks</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">best time to buy and sell stocks II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">best time to buy and sell stocks III</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-iii/</t>
   </si>
 </sst>
 </file>
@@ -257,11 +275,17 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1117,7 +1141,7 @@
       </c>
     </row>
     <row r="33" ht="14.25">
-      <c r="A33" s="3">
+      <c r="A33" s="1">
         <v>46086</v>
       </c>
       <c r="B33" t="s">
@@ -1125,6 +1149,39 @@
       </c>
       <c r="C33" s="2" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="A34" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B34" t="s">
+        <v>67</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="A35" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" ht="14.25">
+      <c r="A36" s="4">
+        <v>46086</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1160,6 +1217,9 @@
     <hyperlink r:id="rId29" ref="C31"/>
     <hyperlink r:id="rId30" ref="C32"/>
     <hyperlink r:id="rId31" ref="C33"/>
+    <hyperlink r:id="rId32" ref="C34"/>
+    <hyperlink r:id="rId33" ref="C35"/>
+    <hyperlink r:id="rId34" ref="C36"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: best time to buy and sell stocks 4
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t>date</t>
   </si>
@@ -235,6 +235,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-iii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">best time to buy and sell stocks IV</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-iv/</t>
   </si>
 </sst>
 </file>
@@ -275,14 +281,13 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -1174,14 +1179,22 @@
       </c>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="4">
+      <c r="A36" s="1">
         <v>46086</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="3" t="s">
         <v>71</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>72</v>
+      </c>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="B37" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1220,6 +1233,7 @@
     <hyperlink r:id="rId32" ref="C34"/>
     <hyperlink r:id="rId33" ref="C35"/>
     <hyperlink r:id="rId34" ref="C36"/>
+    <hyperlink r:id="rId35" ref="C37"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: number of islands
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>date</t>
   </si>
@@ -241,6 +241,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/best-time-to-buy-and-sell-stock-iv/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximal square</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximal-square/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no. of islands</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-islands/description/</t>
   </si>
 </sst>
 </file>
@@ -288,9 +300,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
-    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1190,11 +1200,36 @@
       </c>
     </row>
     <row r="37" ht="14.25">
-      <c r="B37" s="4" t="s">
+      <c r="A37" s="1">
+        <v>46087</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>73</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>74</v>
+      </c>
+    </row>
+    <row r="38" ht="14.25">
+      <c r="A38" s="1">
+        <v>46088</v>
+      </c>
+      <c r="B38" t="s">
+        <v>75</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" ht="14.25">
+      <c r="A39" s="4">
+        <v>46088</v>
+      </c>
+      <c r="B39" t="s">
+        <v>77</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1234,6 +1269,8 @@
     <hyperlink r:id="rId33" ref="C35"/>
     <hyperlink r:id="rId34" ref="C36"/>
     <hyperlink r:id="rId35" ref="C37"/>
+    <hyperlink r:id="rId36" ref="C38"/>
+    <hyperlink r:id="rId37" ref="C39"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: distinct number of islands
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t>date</t>
   </si>
@@ -253,6 +253,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/number-of-islands/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">distinct no. of islands</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/number-of-distinct-islands/1</t>
   </si>
 </sst>
 </file>
@@ -1222,7 +1228,7 @@
       </c>
     </row>
     <row r="39" ht="14.25">
-      <c r="A39" s="4">
+      <c r="A39" s="1">
         <v>46088</v>
       </c>
       <c r="B39" t="s">
@@ -1230,6 +1236,17 @@
       </c>
       <c r="C39" s="2" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="A40" s="4">
+        <v>46088</v>
+      </c>
+      <c r="B40" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1271,6 +1288,7 @@
     <hyperlink r:id="rId35" ref="C37"/>
     <hyperlink r:id="rId36" ref="C38"/>
     <hyperlink r:id="rId37" ref="C39"/>
+    <hyperlink r:id="rId38" ref="C40"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: detect cycle in a directed graph using BFS and DFS
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
   <si>
     <t>date</t>
   </si>
@@ -301,6 +301,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/evaluate-division/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">detect cycle in directed graph</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/detect-cycle-in-a-directed-graph/1</t>
   </si>
 </sst>
 </file>
@@ -341,14 +347,13 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1358,7 +1363,7 @@
       </c>
     </row>
     <row r="47" ht="14.25">
-      <c r="A47" s="4">
+      <c r="A47" s="1">
         <v>46090</v>
       </c>
       <c r="B47" t="s">
@@ -1366,6 +1371,14 @@
       </c>
       <c r="C47" s="2" t="s">
         <v>94</v>
+      </c>
+    </row>
+    <row r="48" ht="14.25">
+      <c r="B48" t="s">
+        <v>95</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1415,6 +1428,7 @@
     <hyperlink r:id="rId43" ref="C45"/>
     <hyperlink r:id="rId44" ref="C46"/>
     <hyperlink r:id="rId45" ref="C47"/>
+    <hyperlink r:id="rId46" ref="C48"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: letter combination of a phone no.
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t>date</t>
   </si>
@@ -349,6 +349,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/word-ladder/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Letter Combination of a Phone No.</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/letter-combinations-of-a-phone-number/</t>
   </si>
 </sst>
 </file>
@@ -1494,7 +1500,7 @@
       </c>
     </row>
     <row r="55" ht="14.25">
-      <c r="A55" s="4">
+      <c r="A55" s="1">
         <v>46095</v>
       </c>
       <c r="B55" t="s">
@@ -1502,6 +1508,17 @@
       </c>
       <c r="C55" s="2" t="s">
         <v>110</v>
+      </c>
+    </row>
+    <row r="56" ht="14.25">
+      <c r="A56" s="4">
+        <v>46096</v>
+      </c>
+      <c r="B56" t="s">
+        <v>111</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -1559,6 +1576,7 @@
     <hyperlink r:id="rId51" ref="C53"/>
     <hyperlink r:id="rId52" ref="C54"/>
     <hyperlink r:id="rId53" ref="C55"/>
+    <hyperlink r:id="rId54" ref="C56"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Invert a binary tree
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="137">
   <si>
     <t>date</t>
   </si>
@@ -421,6 +421,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/same-tree/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">invert binary tree</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/invert-binary-tree/</t>
   </si>
 </sst>
 </file>
@@ -1698,7 +1704,7 @@
       </c>
     </row>
     <row r="67" ht="14.25">
-      <c r="A67" s="4">
+      <c r="A67" s="1">
         <v>46101</v>
       </c>
       <c r="B67" t="s">
@@ -1706,6 +1712,17 @@
       </c>
       <c r="C67" s="2" t="s">
         <v>134</v>
+      </c>
+    </row>
+    <row r="68" ht="14.25">
+      <c r="A68" s="4">
+        <v>46102</v>
+      </c>
+      <c r="B68" t="s">
+        <v>135</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1775,6 +1792,7 @@
     <hyperlink r:id="rId63" ref="C65"/>
     <hyperlink r:id="rId64" ref="C66"/>
     <hyperlink r:id="rId65" ref="C67"/>
+    <hyperlink r:id="rId66" ref="C68"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Binary tree zig-zag level-order traversal
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="175">
   <si>
     <t>date</t>
   </si>
@@ -535,6 +535,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-level-order-traversal/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary Tree Zig-Zag traversal</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/</t>
   </si>
 </sst>
 </file>
@@ -2022,7 +2028,7 @@
       </c>
     </row>
     <row r="86" ht="14.25">
-      <c r="A86" s="5">
+      <c r="A86" s="1">
         <v>46109</v>
       </c>
       <c r="B86" t="s">
@@ -2030,6 +2036,17 @@
       </c>
       <c r="C86" s="2" t="s">
         <v>172</v>
+      </c>
+    </row>
+    <row r="87" ht="14.25">
+      <c r="A87" s="5">
+        <v>46109</v>
+      </c>
+      <c r="B87" t="s">
+        <v>173</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2118,6 +2135,7 @@
     <hyperlink r:id="rId82" ref="C84"/>
     <hyperlink r:id="rId83" ref="C85"/>
     <hyperlink r:id="rId84" ref="C86"/>
+    <hyperlink r:id="rId85" ref="C87"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Min. Abs. Diff. in BST
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="177">
   <si>
     <t>date</t>
   </si>
@@ -541,6 +541,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min abs diff in BST</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/minimum-absolute-difference-in-bst/</t>
   </si>
 </sst>
 </file>
@@ -2039,7 +2045,7 @@
       </c>
     </row>
     <row r="87" ht="14.25">
-      <c r="A87" s="5">
+      <c r="A87" s="1">
         <v>46109</v>
       </c>
       <c r="B87" t="s">
@@ -2047,6 +2053,17 @@
       </c>
       <c r="C87" s="2" t="s">
         <v>174</v>
+      </c>
+    </row>
+    <row r="88" ht="14.25">
+      <c r="A88" s="5">
+        <v>46109</v>
+      </c>
+      <c r="B88" t="s">
+        <v>175</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -2136,6 +2153,7 @@
     <hyperlink r:id="rId83" ref="C85"/>
     <hyperlink r:id="rId84" ref="C86"/>
     <hyperlink r:id="rId85" ref="C87"/>
+    <hyperlink r:id="rId86" ref="C88"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: kth smallest element in BST
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="179">
   <si>
     <t>date</t>
   </si>
@@ -547,6 +547,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/minimum-absolute-difference-in-bst/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kth smallest element in a BST</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/kth-smallest-element-in-a-bst/</t>
   </si>
 </sst>
 </file>
@@ -2056,7 +2062,7 @@
       </c>
     </row>
     <row r="88" ht="14.25">
-      <c r="A88" s="5">
+      <c r="A88" s="1">
         <v>46109</v>
       </c>
       <c r="B88" t="s">
@@ -2064,6 +2070,17 @@
       </c>
       <c r="C88" s="2" t="s">
         <v>176</v>
+      </c>
+    </row>
+    <row r="89" ht="14.25">
+      <c r="A89" s="5">
+        <v>46110</v>
+      </c>
+      <c r="B89" t="s">
+        <v>177</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -2154,6 +2171,7 @@
     <hyperlink r:id="rId84" ref="C86"/>
     <hyperlink r:id="rId85" ref="C87"/>
     <hyperlink r:id="rId86" ref="C88"/>
+    <hyperlink r:id="rId87" ref="C89"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Check if a no. is palindrome or not
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="183">
   <si>
     <t>date</t>
   </si>
@@ -559,6 +559,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/validate-binary-search-tree/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Palindrome Number</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/palindrome-number/</t>
   </si>
 </sst>
 </file>
@@ -2090,7 +2096,7 @@
       </c>
     </row>
     <row r="90" ht="14.25">
-      <c r="A90" s="5">
+      <c r="A90" s="1">
         <v>46110</v>
       </c>
       <c r="B90" t="s">
@@ -2098,6 +2104,17 @@
       </c>
       <c r="C90" s="2" t="s">
         <v>180</v>
+      </c>
+    </row>
+    <row r="91" ht="14.25">
+      <c r="A91" s="5">
+        <v>46111</v>
+      </c>
+      <c r="B91" t="s">
+        <v>181</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -2190,6 +2207,7 @@
     <hyperlink r:id="rId86" ref="C88"/>
     <hyperlink r:id="rId87" ref="C89"/>
     <hyperlink r:id="rId88" ref="C90"/>
+    <hyperlink r:id="rId89" ref="C91"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Count trailing Zeroes in Factorial no.
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="187">
   <si>
     <t>date</t>
   </si>
@@ -571,6 +571,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/plus-one/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factorial Trailing Zeroes</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/factorial-trailing-zeroes/</t>
   </si>
 </sst>
 </file>
@@ -2124,7 +2130,7 @@
       </c>
     </row>
     <row r="92" ht="14.25">
-      <c r="A92" s="5">
+      <c r="A92" s="1">
         <v>46111</v>
       </c>
       <c r="B92" t="s">
@@ -2132,6 +2138,17 @@
       </c>
       <c r="C92" s="2" t="s">
         <v>184</v>
+      </c>
+    </row>
+    <row r="93" ht="14.25">
+      <c r="A93" s="5">
+        <v>46112</v>
+      </c>
+      <c r="B93" t="s">
+        <v>185</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2226,6 +2243,7 @@
     <hyperlink r:id="rId88" ref="C90"/>
     <hyperlink r:id="rId89" ref="C91"/>
     <hyperlink r:id="rId90" ref="C92"/>
+    <hyperlink r:id="rId91" ref="C93"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: compute x to the power n in logn TC
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="191">
   <si>
     <t>date</t>
   </si>
@@ -583,6 +583,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/sqrtx/</t>
+  </si>
+  <si>
+    <t>Pow(x,n)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/powx-n/</t>
   </si>
 </sst>
 </file>
@@ -2158,7 +2164,7 @@
       </c>
     </row>
     <row r="94" ht="14.25">
-      <c r="A94" s="5">
+      <c r="A94" s="1">
         <v>46112</v>
       </c>
       <c r="B94" t="s">
@@ -2166,6 +2172,17 @@
       </c>
       <c r="C94" s="2" t="s">
         <v>188</v>
+      </c>
+    </row>
+    <row r="95" ht="14.25">
+      <c r="A95" s="5">
+        <v>46112</v>
+      </c>
+      <c r="B95" t="s">
+        <v>189</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -2262,6 +2279,7 @@
     <hyperlink r:id="rId90" ref="C92"/>
     <hyperlink r:id="rId91" ref="C93"/>
     <hyperlink r:id="rId92" ref="C94"/>
+    <hyperlink r:id="rId93" ref="C95"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: max points on a line
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="193">
   <si>
     <t>date</t>
   </si>
@@ -589,6 +589,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/powx-n/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max. points on a line</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/max-points-on-a-line/</t>
   </si>
 </sst>
 </file>
@@ -2175,7 +2181,7 @@
       </c>
     </row>
     <row r="95" ht="14.25">
-      <c r="A95" s="5">
+      <c r="A95" s="1">
         <v>46112</v>
       </c>
       <c r="B95" t="s">
@@ -2183,6 +2189,17 @@
       </c>
       <c r="C95" s="2" t="s">
         <v>190</v>
+      </c>
+    </row>
+    <row r="96" ht="14.25">
+      <c r="A96" s="5">
+        <v>46113</v>
+      </c>
+      <c r="B96" t="s">
+        <v>191</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2280,6 +2297,7 @@
     <hyperlink r:id="rId91" ref="C93"/>
     <hyperlink r:id="rId92" ref="C94"/>
     <hyperlink r:id="rId93" ref="C95"/>
+    <hyperlink r:id="rId94" ref="C96"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: bitwise and of nos. in a range
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203">
   <si>
     <t>date</t>
   </si>
@@ -619,6 +619,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/single-number-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitwise and of numbers in a range</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/bitwise-and-of-numbers-range/</t>
   </si>
 </sst>
 </file>
@@ -2260,7 +2266,7 @@
       </c>
     </row>
     <row r="100" ht="14.25">
-      <c r="A100" s="5">
+      <c r="A100" s="1">
         <v>46114</v>
       </c>
       <c r="B100" t="s">
@@ -2268,6 +2274,17 @@
       </c>
       <c r="C100" s="2" t="s">
         <v>200</v>
+      </c>
+    </row>
+    <row r="101" ht="14.25">
+      <c r="A101" s="5">
+        <v>46114</v>
+      </c>
+      <c r="B101" t="s">
+        <v>201</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -2370,6 +2387,7 @@
     <hyperlink r:id="rId96" ref="C98"/>
     <hyperlink r:id="rId97" ref="C99"/>
     <hyperlink r:id="rId98" ref="C100"/>
+    <hyperlink r:id="rId99" ref="C101"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: binary search if target is present or not
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="215">
   <si>
     <t>date</t>
   </si>
@@ -655,6 +655,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/find-median-from-data-stream/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">search insert position</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/search-insert-position/</t>
   </si>
 </sst>
 </file>
@@ -2362,7 +2368,7 @@
       </c>
     </row>
     <row r="106" ht="14.25">
-      <c r="A106" s="5">
+      <c r="A106" s="1">
         <v>46116</v>
       </c>
       <c r="B106" t="s">
@@ -2370,6 +2376,17 @@
       </c>
       <c r="C106" s="2" t="s">
         <v>212</v>
+      </c>
+    </row>
+    <row r="107" ht="14.25">
+      <c r="A107" s="5">
+        <v>46116</v>
+      </c>
+      <c r="B107" t="s">
+        <v>213</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -2478,6 +2495,7 @@
     <hyperlink r:id="rId102" ref="C104"/>
     <hyperlink r:id="rId103" ref="C105"/>
     <hyperlink r:id="rId104" ref="C106"/>
+    <hyperlink r:id="rId105" ref="C107"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: search in a 2d matrix
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217">
   <si>
     <t>date</t>
   </si>
@@ -661,6 +661,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/search-insert-position/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">search in a 2D matrix</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/search-a-2d-matrix/</t>
   </si>
 </sst>
 </file>
@@ -2379,7 +2385,7 @@
       </c>
     </row>
     <row r="107" ht="14.25">
-      <c r="A107" s="5">
+      <c r="A107" s="1">
         <v>46116</v>
       </c>
       <c r="B107" t="s">
@@ -2387,6 +2393,17 @@
       </c>
       <c r="C107" s="2" t="s">
         <v>214</v>
+      </c>
+    </row>
+    <row r="108" ht="14.25">
+      <c r="A108" s="5">
+        <v>46117</v>
+      </c>
+      <c r="B108" t="s">
+        <v>215</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2496,6 +2513,7 @@
     <hyperlink r:id="rId103" ref="C105"/>
     <hyperlink r:id="rId104" ref="C106"/>
     <hyperlink r:id="rId105" ref="C107"/>
+    <hyperlink r:id="rId106" ref="C108"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: next greater element II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="227">
   <si>
     <t>date</t>
   </si>
@@ -691,6 +691,12 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/next-larger-element-1587115620/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">next greater element II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/next-greater-element-ii/</t>
   </si>
 </sst>
 </file>
@@ -2453,7 +2459,7 @@
       </c>
     </row>
     <row r="111" ht="14.25">
-      <c r="A111" s="5">
+      <c r="A111" s="1">
         <v>46118</v>
       </c>
       <c r="B111" t="s">
@@ -2464,7 +2470,7 @@
       </c>
     </row>
     <row r="112" ht="14.25">
-      <c r="A112" s="5">
+      <c r="A112" s="1">
         <v>46118</v>
       </c>
       <c r="B112" t="s">
@@ -2472,6 +2478,17 @@
       </c>
       <c r="C112" s="2" t="s">
         <v>224</v>
+      </c>
+    </row>
+    <row r="113" ht="14.25">
+      <c r="A113" s="5">
+        <v>46118</v>
+      </c>
+      <c r="B113" t="s">
+        <v>225</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -2586,6 +2603,7 @@
     <hyperlink r:id="rId108" ref="C110"/>
     <hyperlink r:id="rId109" ref="C111"/>
     <hyperlink r:id="rId110" ref="C112"/>
+    <hyperlink r:id="rId111" ref="C113"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: search in rotated-sorted array
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="229">
   <si>
     <t>date</t>
   </si>
@@ -697,6 +697,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/next-greater-element-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">search in sorted rotated array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/search-in-rotated-sorted-array</t>
   </si>
 </sst>
 </file>
@@ -2481,7 +2487,7 @@
       </c>
     </row>
     <row r="113" ht="14.25">
-      <c r="A113" s="5">
+      <c r="A113" s="1">
         <v>46118</v>
       </c>
       <c r="B113" t="s">
@@ -2489,6 +2495,17 @@
       </c>
       <c r="C113" s="2" t="s">
         <v>226</v>
+      </c>
+    </row>
+    <row r="114" ht="14.25">
+      <c r="A114" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B114" t="s">
+        <v>227</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -2604,6 +2621,7 @@
     <hyperlink r:id="rId109" ref="C111"/>
     <hyperlink r:id="rId110" ref="C112"/>
     <hyperlink r:id="rId111" ref="C113"/>
+    <hyperlink r:id="rId112" ref="C114"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: find min. in rotated sorted array
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="235">
   <si>
     <t>date</t>
   </si>
@@ -715,6 +715,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/lru-cache/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">find min. in rotated sorted array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/</t>
   </si>
 </sst>
 </file>
@@ -2532,7 +2538,7 @@
       </c>
     </row>
     <row r="116" ht="14.25">
-      <c r="A116" s="5">
+      <c r="A116" s="1">
         <v>46120</v>
       </c>
       <c r="B116" t="s">
@@ -2540,6 +2546,17 @@
       </c>
       <c r="C116" s="2" t="s">
         <v>232</v>
+      </c>
+    </row>
+    <row r="117" ht="14.25">
+      <c r="A117" s="5">
+        <v>46120</v>
+      </c>
+      <c r="B117" t="s">
+        <v>233</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -2658,6 +2675,7 @@
     <hyperlink r:id="rId112" ref="C114"/>
     <hyperlink r:id="rId113" ref="C115"/>
     <hyperlink r:id="rId114" ref="C116"/>
+    <hyperlink r:id="rId115" ref="C117"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: median of 2 sorted arrays
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="241">
   <si>
     <t>date</t>
   </si>
@@ -733,6 +733,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/rotate-array/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median of 2 sorted arrays</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/median-of-two-sorted-arrays/</t>
   </si>
 </sst>
 </file>
@@ -2583,7 +2589,7 @@
       </c>
     </row>
     <row r="119" ht="14.25">
-      <c r="A119" s="5">
+      <c r="A119" s="1">
         <v>46120</v>
       </c>
       <c r="B119" t="s">
@@ -2591,6 +2597,17 @@
       </c>
       <c r="C119" s="2" t="s">
         <v>238</v>
+      </c>
+    </row>
+    <row r="120" ht="14.25">
+      <c r="A120" s="5">
+        <v>46121</v>
+      </c>
+      <c r="B120" t="s">
+        <v>239</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -2712,6 +2729,7 @@
     <hyperlink r:id="rId115" ref="C117"/>
     <hyperlink r:id="rId116" ref="C118"/>
     <hyperlink r:id="rId117" ref="C119"/>
+    <hyperlink r:id="rId118" ref="C120"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Max. sum circular subarray
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="245">
   <si>
     <t>date</t>
   </si>
@@ -745,6 +745,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/maximum-subarray</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max sum circular subarray</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-sum-circular-subarray/</t>
   </si>
 </sst>
 </file>
@@ -785,7 +791,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -794,6 +800,9 @@
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2617,7 +2626,7 @@
       </c>
     </row>
     <row r="121" ht="14.25">
-      <c r="A121" s="5">
+      <c r="A121" s="1">
         <v>46122</v>
       </c>
       <c r="B121" t="s">
@@ -2625,6 +2634,17 @@
       </c>
       <c r="C121" s="2" t="s">
         <v>242</v>
+      </c>
+    </row>
+    <row r="122" ht="14.25">
+      <c r="A122" s="5">
+        <v>46123</v>
+      </c>
+      <c r="B122" t="s">
+        <v>243</v>
+      </c>
+      <c r="C122" s="6" t="s">
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -2748,6 +2768,7 @@
     <hyperlink r:id="rId117" ref="C119"/>
     <hyperlink r:id="rId118" ref="C120"/>
     <hyperlink r:id="rId119" ref="C121"/>
+    <hyperlink r:id="rId120" ref="C122"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: construct quad tree
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="251">
   <si>
     <t>date</t>
   </si>
@@ -763,6 +763,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/sort-list/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">construct quad tree</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/construct-quad-tree/</t>
   </si>
 </sst>
 </file>
@@ -2671,7 +2677,7 @@
       </c>
     </row>
     <row r="124" ht="14.25">
-      <c r="A124" s="6">
+      <c r="A124" s="1">
         <v>46124</v>
       </c>
       <c r="B124" t="s">
@@ -2679,6 +2685,17 @@
       </c>
       <c r="C124" s="2" t="s">
         <v>248</v>
+      </c>
+    </row>
+    <row r="125" ht="14.25">
+      <c r="A125" s="6">
+        <v>46124</v>
+      </c>
+      <c r="B125" t="s">
+        <v>249</v>
+      </c>
+      <c r="C125" s="2" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -2805,6 +2822,7 @@
     <hyperlink r:id="rId120" ref="C122"/>
     <hyperlink r:id="rId121" ref="C123"/>
     <hyperlink r:id="rId122" ref="C124"/>
+    <hyperlink r:id="rId123" ref="C125"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: diameter of binary tree
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="293">
   <si>
     <t>date</t>
   </si>
@@ -889,6 +889,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/valid-anagram/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diameter of a binary tree</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/diameter-of-binary-tree/</t>
   </si>
 </sst>
 </file>
@@ -3028,7 +3034,7 @@
       </c>
     </row>
     <row r="145" ht="14.25">
-      <c r="A145" s="6">
+      <c r="A145" s="1">
         <v>46142</v>
       </c>
       <c r="B145" t="s">
@@ -3036,6 +3042,17 @@
       </c>
       <c r="C145" s="2" t="s">
         <v>290</v>
+      </c>
+    </row>
+    <row r="146" ht="14.25">
+      <c r="A146" s="6">
+        <v>46143</v>
+      </c>
+      <c r="B146" t="s">
+        <v>291</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -3183,6 +3200,7 @@
     <hyperlink r:id="rId141" ref="C143"/>
     <hyperlink r:id="rId142" ref="C144"/>
     <hyperlink r:id="rId143" ref="C145"/>
+    <hyperlink r:id="rId144" ref="C146"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>